<commit_message>
Updated IND_grids_kan60 model - 2026-09-28 15:04
</commit_message>
<xml_diff>
--- a/VerveStacks_IND_grids_kan60/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_IND_grids_kan60/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IND_grids_kan60\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B8A4279-8948-4BC6-9EFA-C1FDEA1A1486}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40AA704B-BBC1-4E4B-B52A-AFE23E233F87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1103" yWindow="1103" windowWidth="21600" windowHeight="12772" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3675" yWindow="3675" windowWidth="21600" windowHeight="11423" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap" sheetId="70" r:id="rId1"/>
@@ -4615,7 +4615,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D655B332-F3A5-4E95-8D69-083D88D286FD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB253438-C560-409F-ADF7-D8E5D3CFFFAA}">
   <dimension ref="B9:L273"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -34693,7 +34693,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{747231A5-264E-405A-AE2E-278DE4466F8F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D2A29E4-4365-47F2-A0FD-3157C5D4135B}">
   <dimension ref="B9:H273"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>